<commit_message>
Ship the next shift of the day, and keep listing-error and later ship-by orders out of the wrong piles.
Sorter writes the next shift on each run, takes only due orders from the 3rd shift on, and skips warehouse-OOS plus the personalised listing-error tag. Custom matches as a whole word. Each DTF file starts with a Batch Summary.
</commit_message>
<xml_diff>
--- a/Order Grouping Sorter/order-grouping-progress.xlsx
+++ b/Order Grouping Sorter/order-grouping-progress.xlsx
@@ -715,7 +715,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Order grouping  ·  2026-10-09</t>
+          <t>Order grouping  ·  2026-10-14</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -813,7 +813,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>testing: every --run is 1st Shift; production later S2 / S3</t>
+          <t>nth --run of the day = nth shift (S1, S2, S3, …)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -904,8 +904,9 @@
       <c r="B12" s="13" t="inlineStr">
         <is>
           <t>2. Skip
-post-order-designs
-and 00000-Warehouse OOS</t>
+post-order-designs,
+00000-Warehouse OOS,
+1006 listing error</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
@@ -1002,7 +1003,7 @@
       </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>Testing: filename field 1 S1 (after optional B-batch prefix) and Input 1st Shift every --run. Hashim #037: order volume &gt; 300 splits today vs later dates; do not dump into Shift 2/3. Blank ship-by → today (in awaiting_shipment → pull today; 2026-09-24). Production later: nth run = nth shift</t>
+          <t>Nth --run of the day = nth shift (S1, S2, S3). 3rd shift and later write due orders only; later ship-by stays in awaiting_shipment. Hashim #037: order volume &gt; 300 splits today vs later on 1st/2nd. Blank ship-by → today.</t>
         </is>
       </c>
       <c r="E17" s="19" t="inlineStr">
@@ -1164,7 +1165,7 @@
       </c>
       <c r="D23" s="18" t="inlineStr">
         <is>
-          <t>CL Customise. Mixed P vs R in one order: majority printed units; tie → readymade (not unmatched)</t>
+          <t>CL Customise. Item Name Custom / Customisable / Customised are whole words (2026-10-14); Personali stays a substring. Mixed P vs R: majority printed units; tie → readymade</t>
         </is>
       </c>
       <c r="E23" s="19" t="inlineStr">
@@ -1338,7 +1339,7 @@
     <row r="30">
       <c r="A30" s="23" t="inlineStr">
         <is>
-          <t>Fixed batches first (B10…B8050, row order = priority), then plain B2000/B2100/B2200/B2500/B2600/… and printed leftover B1/B2/… skipping reserved. Hashim #037: orders &gt; 300 split today vs later. Testing: --run rewrites 1st Shift. Packing PIN: B100-S1-1 Item 1 (batch+shift only).</t>
+          <t>Fixed batches first (B10…B8050, row order = priority), then plain B2000/B2100/B2200/B2500/B2600/… and printed leftover B1/B2/… skipping reserved. Hashim #037: orders &gt; 300 split today vs later on 1st/2nd. Nth --run = nth shift. 3rd+ is due orders only. Packing PIN: B100-S1-1 Item 1 (batch+shift only).</t>
         </is>
       </c>
       <c r="B30" s="2" t="n"/>
@@ -1933,7 +1934,7 @@
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
         <is>
-          <t>Plain Database.xlsx</t>
+          <t>Plain Database.csv</t>
         </is>
       </c>
       <c r="B19" s="17" t="inlineStr">

</xml_diff>

<commit_message>
Ship sorter shift gates, catalog fill locks, and shipping reprint reuse.
Lock 3rd+ shift ship-by/tag rules, print-size and UID fill policy, and Shipping convert/reprint/Batch Summary so the warehouse keeps matching how the floor already runs.
</commit_message>
<xml_diff>
--- a/Order Grouping Sorter/order-grouping-progress.xlsx
+++ b/Order Grouping Sorter/order-grouping-progress.xlsx
@@ -715,7 +715,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Order grouping  ·  2026-10-14</t>
+          <t>Order grouping  ·  2026-10-22</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -830,7 +830,7 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Fixed batches: B40/B80/B100/B1050/B3700/…. Leftover: B1/B2/… (skip reserved). Filename keeps full 6 fields. Packing PIN uses B100-S1-1 Item 1 only. Shift folder stays 1st/2nd/3rd. Amazon stays in own. MAS Clothing → fawad (match only).</t>
+          <t>Fixed batches: B40/B80/B100/B1050/B6000/B3700/…. Leftover: B1/B2/… (skip reserved). Filename keeps full 6 fields. Packing PIN uses B100-S1-1 Item 1 only. Shift folder stays 1st/2nd/3rd. Amazon stays in own. MAS Clothing → fawad (match only).</t>
         </is>
       </c>
       <c r="C6" s="2" t="n"/>
@@ -850,7 +850,7 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>filename is only:  RESEND     Exact tag 1014-ALL-RESEND only (not 1015 / 1016 / 1017). Wins even if ship-by is blank.</t>
+          <t>1014-ALL-RESEND → B9000 ready-made tees, B9050 personalised tees, B9040 Gildan, B9100 / B9150 iron-on, B9200 other. Catalog-miss stays RESEND. Not held for a missing 1004 tag (2026-10-18).</t>
         </is>
       </c>
       <c r="C8" s="2" t="n"/>
@@ -870,7 +870,7 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>filename is only:  UNMATCHED     No definite match. Floor handles this run; then investigate and tighten so the next run matches. Same order stays together.</t>
+          <t>filename is only:  UNMATCHED     No definite match. Chat run does not seed the catalog (2026-10-20). add unmatched is a separate script. Same order stays together.</t>
         </is>
       </c>
       <c r="C9" s="2" t="n"/>
@@ -912,7 +912,7 @@
       <c r="C12" s="13" t="inlineStr">
         <is>
           <t>3. Resend tag?
-→ file “RESEND”</t>
+→ B9040–B9200</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>Nth --run of the day = nth shift (S1, S2, S3). 3rd shift and later write due orders only; later ship-by stays in awaiting_shipment. Hashim #037: order volume &gt; 300 splits today vs later on 1st/2nd. Blank ship-by → today.</t>
+          <t>Nth --run of the day = nth shift (S1, S2, S3). 3rd shift and later write overdue, blank, and the run-day ship-by, plus tag 1004- Personalised Design-Ready- when ship-by is later (locked 2026-10-22). A later ship-by without that tag stays out.  Hashim #037: order volume &gt; 300 splits today vs later on 1st/2nd. Blank ship-by → today.</t>
         </is>
       </c>
       <c r="E17" s="19" t="inlineStr">
@@ -1339,7 +1339,7 @@
     <row r="30">
       <c r="A30" s="23" t="inlineStr">
         <is>
-          <t>Fixed batches first (B10…B8050, row order = priority), then plain B2000/B2100/B2200/B2500/B2600/… and printed leftover B1/B2/… skipping reserved. Hashim #037: orders &gt; 300 split today vs later on 1st/2nd. Nth --run = nth shift. 3rd+ is due orders only. Packing PIN: B100-S1-1 Item 1 (batch+shift only).</t>
+          <t>Fixed batches first (B10 international under resend, B700 UK UV, B6000/B6010 UK plain bags, B6020/B6030/B6050/B6060 UK printed bags, B40 any Gildan tee, B8000/B8050 prime FOTL, B7000/B3000 odd items last). Then plain B2000/… and printed leftover B1/B2/… skipping reserved. Nth --run = nth shift. 3rd+ writes overdue, blank, and the run-day ship-by, plus tag 1004- Personalised Design-Ready- when ship-by is later (locked 2026-10-22). A later ship-by without that tag stays out.  Packing PIN: B100-S1-1 Item 1.</t>
         </is>
       </c>
       <c r="B30" s="2" t="n"/>

</xml_diff>